<commit_message>
updated and cleaned code to remove masters only institutions from calculation of PCR values
</commit_message>
<xml_diff>
--- a/PRC_National_dataset test.xlsx
+++ b/PRC_National_dataset test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/co25936/Desktop/PER/IPEDS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{29A08B0D-83FC-0D47-8590-70E9503644C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61AC618-1AD8-634D-A11F-7A949148D27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="38400" windowHeight="17620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -221,7 +221,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -527,10 +527,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:V1098"/>
+  <dimension ref="A1:AD1098"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -561,20 +561,20 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="T1" t="s">
         <v>32</v>
       </c>
-      <c r="M1" t="s">
+      <c r="U1" t="s">
         <v>33</v>
       </c>
-      <c r="N1" t="s">
+      <c r="V1" t="s">
         <v>34</v>
       </c>
-      <c r="O1" t="s">
+      <c r="W1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2010</v>
       </c>
@@ -600,7 +600,7 @@
         <v>12812</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -632,19 +632,30 @@
         <v>1.049406806119263</v>
       </c>
       <c r="K3" s="3"/>
-      <c r="L3">
+      <c r="L3" s="3">
         <f>(E8+E9+E10)/(G2+G3+G4)</f>
         <v>0.63092424430899363</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3">
+        <f>(E8+E9+E10)/(G2+G3+G4)</f>
+        <v>0.63092424430899363</v>
+      </c>
+      <c r="U3">
         <f>(H3+E3-G3)/H2</f>
         <v>0.93139244458320325</v>
       </c>
-      <c r="N3" t="s">
+      <c r="V3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2012</v>
       </c>
@@ -676,16 +687,27 @@
         <v>1.046905884141706</v>
       </c>
       <c r="K4" s="3"/>
-      <c r="L4">
+      <c r="L4" s="3">
+        <f t="shared" ref="L4:L67" si="0">(E9+E10+E11)/(G3+G4+G5)</f>
+        <v>0.63227155331447549</v>
+      </c>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4">
         <f>(E9+E10+E11)/(G3+G4+G5)</f>
         <v>0.63227155331447549</v>
       </c>
-      <c r="M4">
+      <c r="U4">
         <f>(H4+E4-G4)/H3</f>
         <v>0.92222897977801432</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -717,16 +739,27 @@
         <v>1.063950411973694</v>
       </c>
       <c r="K5" s="3"/>
-      <c r="L5">
-        <f t="shared" ref="L4:L5" si="0">(E10+E11+E12)/(G4+G5+G6)</f>
+      <c r="L5" s="3">
+        <f t="shared" si="0"/>
         <v>0.62905413737822169</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5">
+        <f>(E10+E11+E12)/(G4+G5+G6)</f>
+        <v>0.62905413737822169</v>
+      </c>
+      <c r="U5">
         <f>(H5+E5-G5)/H4</f>
         <v>0.93400861743140073</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -757,8 +790,12 @@
       <c r="J6">
         <v>1.0691702538221759</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="L6" s="3">
+        <f t="shared" si="0"/>
+        <v>0.60389217937870177</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2015</v>
       </c>
@@ -789,20 +826,24 @@
       <c r="J7">
         <v>1.032928942807626</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="3">
+        <f t="shared" si="0"/>
+        <v>0.60497204710360419</v>
+      </c>
+      <c r="T7" t="s">
         <v>23</v>
       </c>
-      <c r="O7" t="s">
+      <c r="W7" t="s">
         <v>24</v>
       </c>
-      <c r="R7" t="s">
+      <c r="Z7" t="s">
         <v>25</v>
       </c>
-      <c r="V7" s="2" t="s">
+      <c r="AD7" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2016</v>
       </c>
@@ -833,11 +874,15 @@
       <c r="J8">
         <v>1.0495628928545631</v>
       </c>
-      <c r="V8" s="2" t="s">
+      <c r="L8" s="3">
+        <f t="shared" si="0"/>
+        <v>0.61846547910117589</v>
+      </c>
+      <c r="AD8" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2017</v>
       </c>
@@ -865,35 +910,39 @@
       <c r="J9">
         <v>1.0109616342800201</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="3">
+        <f t="shared" si="0"/>
+        <v>0.55202477916714465</v>
+      </c>
+      <c r="T9">
         <f>H51+H760</f>
         <v>13762</v>
       </c>
-      <c r="M9">
-        <f>H9-L9</f>
-        <v>0</v>
-      </c>
-      <c r="O9">
+      <c r="U9">
+        <f>H9-T9</f>
+        <v>0</v>
+      </c>
+      <c r="W9">
         <f>H93+H107+H121+H135+H149+H163+H177+H191</f>
         <v>13739</v>
       </c>
-      <c r="P9">
-        <f>H9-O9</f>
+      <c r="X9">
+        <f>H9-W9</f>
         <v>23</v>
       </c>
-      <c r="R9">
+      <c r="Z9">
         <f>H23+H37</f>
         <v>13762</v>
       </c>
-      <c r="S9">
-        <f>H9-R9</f>
-        <v>0</v>
-      </c>
-      <c r="V9" s="2" t="s">
+      <c r="AA9">
+        <f>H9-Z9</f>
+        <v>0</v>
+      </c>
+      <c r="AD9" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -921,35 +970,39 @@
       <c r="J10">
         <v>1.0812381921232379</v>
       </c>
-      <c r="L10">
-        <f t="shared" ref="L10:L15" si="1">H52+H761</f>
+      <c r="L10" s="3">
+        <f t="shared" si="0"/>
+        <v>0.48169622555707142</v>
+      </c>
+      <c r="T10">
+        <f t="shared" ref="T10:T15" si="1">H52+H761</f>
         <v>14259</v>
       </c>
-      <c r="M10">
-        <f t="shared" ref="M10:M15" si="2">H10-L10</f>
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <f t="shared" ref="O10:O15" si="3">H94+H108+H122+H136+H150+H164+H178+H192</f>
+      <c r="U10">
+        <f t="shared" ref="U10:U15" si="2">H10-T10</f>
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <f t="shared" ref="W10:W15" si="3">H94+H108+H122+H136+H150+H164+H178+H192</f>
         <v>14236</v>
       </c>
-      <c r="P10">
-        <f t="shared" ref="P10:P15" si="4">H10-O10</f>
+      <c r="X10">
+        <f t="shared" ref="X10:X15" si="4">H10-W10</f>
         <v>23</v>
       </c>
-      <c r="R10">
-        <f t="shared" ref="R10:R15" si="5">H24+H38</f>
+      <c r="Z10">
+        <f t="shared" ref="Z10:Z15" si="5">H24+H38</f>
         <v>14259</v>
       </c>
-      <c r="S10">
-        <f t="shared" ref="S10:S15" si="6">H10-R10</f>
-        <v>0</v>
-      </c>
-      <c r="V10" s="2" t="s">
+      <c r="AA10">
+        <f t="shared" ref="AA10:AA15" si="6">H10-Z10</f>
+        <v>0</v>
+      </c>
+      <c r="AD10" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2019</v>
       </c>
@@ -977,35 +1030,39 @@
       <c r="J11">
         <v>1.0319096710849289</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="3">
+        <f t="shared" si="0"/>
+        <v>0.43537657400807794</v>
+      </c>
+      <c r="T11">
         <f t="shared" si="1"/>
         <v>14234</v>
       </c>
-      <c r="M11">
+      <c r="U11">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O11">
+      <c r="W11">
         <f t="shared" si="3"/>
         <v>14214</v>
       </c>
-      <c r="P11">
+      <c r="X11">
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="R11">
+      <c r="Z11">
         <f t="shared" si="5"/>
         <v>14234</v>
       </c>
-      <c r="S11">
+      <c r="AA11">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="V11" s="2" t="s">
+      <c r="AD11" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -1033,35 +1090,39 @@
       <c r="J12">
         <v>1.041379794857384</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="3">
+        <f t="shared" si="0"/>
+        <v>0.44926340601060694</v>
+      </c>
+      <c r="T12">
         <f t="shared" si="1"/>
         <v>13912</v>
       </c>
-      <c r="M12">
+      <c r="U12">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O12">
+      <c r="W12">
         <f t="shared" si="3"/>
         <v>13890</v>
       </c>
-      <c r="P12">
+      <c r="X12">
         <f t="shared" si="4"/>
         <v>22</v>
       </c>
-      <c r="R12">
+      <c r="Z12">
         <f t="shared" si="5"/>
         <v>13912</v>
       </c>
-      <c r="S12">
+      <c r="AA12">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="V12" s="2" t="s">
+      <c r="AD12" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -1089,32 +1150,36 @@
       <c r="J13">
         <v>1.067567567567568</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="3">
+        <f t="shared" si="0"/>
+        <v>0.45686113393590799</v>
+      </c>
+      <c r="T13">
         <f t="shared" si="1"/>
         <v>14661</v>
       </c>
-      <c r="M13">
+      <c r="U13">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O13">
+      <c r="W13">
         <f t="shared" si="3"/>
         <v>14644</v>
       </c>
-      <c r="P13">
+      <c r="X13">
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
-      <c r="R13">
+      <c r="Z13">
         <f t="shared" si="5"/>
         <v>14661</v>
       </c>
-      <c r="S13">
+      <c r="AA13">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -1142,32 +1207,36 @@
       <c r="J14">
         <v>1.0394925312052381</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="3">
+        <f t="shared" si="0"/>
+        <v>0.43275691155413593</v>
+      </c>
+      <c r="T14">
         <f t="shared" si="1"/>
         <v>14650</v>
       </c>
-      <c r="M14">
+      <c r="U14">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O14">
+      <c r="W14">
         <f t="shared" si="3"/>
         <v>14635</v>
       </c>
-      <c r="P14">
+      <c r="X14">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
-      <c r="R14">
+      <c r="Z14">
         <f t="shared" si="5"/>
         <v>14650</v>
       </c>
-      <c r="S14">
+      <c r="AA14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -1195,32 +1264,36 @@
       <c r="J15">
         <v>1.0615699658703071</v>
       </c>
-      <c r="L15">
+      <c r="L15" s="3">
+        <f t="shared" si="0"/>
+        <v>0.49461833477669181</v>
+      </c>
+      <c r="T15">
         <f t="shared" si="1"/>
         <v>14978</v>
       </c>
-      <c r="M15">
+      <c r="U15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O15">
+      <c r="W15">
         <f t="shared" si="3"/>
         <v>14965</v>
       </c>
-      <c r="P15">
+      <c r="X15">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="R15">
+      <c r="Z15">
         <f t="shared" si="5"/>
         <v>14978</v>
       </c>
-      <c r="S15">
+      <c r="AA15">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2010</v>
       </c>
@@ -1245,8 +1318,12 @@
       <c r="H16">
         <v>10250</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L16" s="3">
+        <f t="shared" si="0"/>
+        <v>0.55735012318642208</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2011</v>
       </c>
@@ -1277,8 +1354,12 @@
       <c r="J17">
         <v>1.0505365853658539</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L17" s="3">
+        <f t="shared" si="0"/>
+        <v>0.63861617578307617</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2012</v>
       </c>
@@ -1309,8 +1390,12 @@
       <c r="J18">
         <v>1.0428218761868591</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L18" s="3">
+        <f t="shared" si="0"/>
+        <v>0.63516213308744429</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2013</v>
       </c>
@@ -1341,8 +1426,12 @@
       <c r="J19">
         <v>1.0693537704607821</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L19" s="3">
+        <f t="shared" si="0"/>
+        <v>0.62526997840172782</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2014</v>
       </c>
@@ -1373,8 +1462,12 @@
       <c r="J20">
         <v>1.066204345815996</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L20" s="3">
+        <f t="shared" si="0"/>
+        <v>0.60766423357664234</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2015</v>
       </c>
@@ -1405,8 +1498,12 @@
       <c r="J21">
         <v>1.0316615551145589</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L21" s="3">
+        <f t="shared" si="0"/>
+        <v>0.6111027304269121</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2016</v>
       </c>
@@ -1437,8 +1534,12 @@
       <c r="J22">
         <v>1.046082949308756</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L22" s="3">
+        <f t="shared" si="0"/>
+        <v>0.62579783286329227</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2017</v>
       </c>
@@ -1466,8 +1567,12 @@
       <c r="J23">
         <v>1.008593680064453</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L23" s="3">
+        <f t="shared" si="0"/>
+        <v>0.46347533304055044</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2018</v>
       </c>
@@ -1495,8 +1600,12 @@
       <c r="J24">
         <v>1.072485071198898</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L24" s="3">
+        <f t="shared" si="0"/>
+        <v>0.28961114335461402</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2019</v>
       </c>
@@ -1524,8 +1633,12 @@
       <c r="J25">
         <v>1.0340433116478029</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L25" s="3">
+        <f t="shared" si="0"/>
+        <v>0.12769866789159393</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2020</v>
       </c>
@@ -1553,8 +1666,12 @@
       <c r="J26">
         <v>1.0376920328688819</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L26" s="3">
+        <f t="shared" si="0"/>
+        <v>0.13811462574381458</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2021</v>
       </c>
@@ -1582,8 +1699,12 @@
       <c r="J27">
         <v>1.0628460686600221</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L27" s="3">
+        <f t="shared" si="0"/>
+        <v>0.14632187600385479</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>2022</v>
       </c>
@@ -1611,8 +1732,12 @@
       <c r="J28">
         <v>1.042278753135077</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L28" s="3">
+        <f t="shared" si="0"/>
+        <v>0.14222425908952033</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>2023</v>
       </c>
@@ -1640,8 +1765,12 @@
       <c r="J29">
         <v>1.0666787790697669</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L29" s="3">
+        <f t="shared" si="0"/>
+        <v>0.19267188143268835</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2010</v>
       </c>
@@ -1666,8 +1795,12 @@
       <c r="H30">
         <v>2562</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L30" s="3">
+        <f t="shared" si="0"/>
+        <v>0.28554070473876064</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>2011</v>
       </c>
@@ -1698,8 +1831,12 @@
       <c r="J31">
         <v>1.0448868071818891</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L31" s="3">
+        <f t="shared" si="0"/>
+        <v>0.6004932182490752</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>2012</v>
       </c>
@@ -1730,8 +1867,12 @@
       <c r="J32">
         <v>1.063310450038139</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L32" s="3">
+        <f t="shared" si="0"/>
+        <v>0.62068965517241381</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>2013</v>
       </c>
@@ -1762,8 +1903,12 @@
       <c r="J33">
         <v>1.042481203007519</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L33" s="3">
+        <f t="shared" si="0"/>
+        <v>0.64413030116779346</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>2014</v>
       </c>
@@ -1794,8 +1939,12 @@
       <c r="J34">
         <v>1.0812335464460321</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L34" s="3">
+        <f t="shared" si="0"/>
+        <v>0.58927519151443719</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>2015</v>
       </c>
@@ -1826,8 +1975,12 @@
       <c r="J35">
         <v>1.0380159304851559</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L35" s="3">
+        <f t="shared" si="0"/>
+        <v>0.58211473565804273</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>2016</v>
       </c>
@@ -1858,8 +2011,12 @@
       <c r="J36">
         <v>1.0634462869502519</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L36" s="3">
+        <f t="shared" si="0"/>
+        <v>0.59179265658747304</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>2017</v>
       </c>
@@ -1887,8 +2044,12 @@
       <c r="J37">
         <v>1.0201528839471861</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L37" s="3">
+        <f t="shared" si="0"/>
+        <v>1.1452810180275717</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>2018</v>
       </c>
@@ -1916,8 +2077,12 @@
       <c r="J38">
         <v>1.1143552311435521</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L38" s="3">
+        <f t="shared" si="0"/>
+        <v>1.7232142857142858</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>2019</v>
       </c>
@@ -1945,8 +2110,12 @@
       <c r="J39">
         <v>1.02402896642528</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L39" s="3">
+        <f t="shared" si="0"/>
+        <v>2.3842077371489134</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2020</v>
       </c>
@@ -1974,8 +2143,12 @@
       <c r="J40">
         <v>1.0549703752468731</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L40" s="3">
+        <f t="shared" si="0"/>
+        <v>2.2363030014292522</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>2021</v>
       </c>
@@ -2003,8 +2176,12 @@
       <c r="J41">
         <v>1.0842002600780229</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L41" s="3">
+        <f t="shared" si="0"/>
+        <v>2.094635848233755</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>2022</v>
       </c>
@@ -2032,8 +2209,12 @@
       <c r="J42">
         <v>1.030597655132971</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L42" s="3">
+        <f t="shared" si="0"/>
+        <v>1.9186735096723253</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>2023</v>
       </c>
@@ -2061,8 +2242,12 @@
       <c r="J43">
         <v>1.0461285008237231</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L43" s="3">
+        <f t="shared" si="0"/>
+        <v>2.940405244338498</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>2010</v>
       </c>
@@ -2087,8 +2272,12 @@
       <c r="H44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L44" s="3">
+        <f t="shared" si="0"/>
+        <v>5.8688524590163933</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>2011</v>
       </c>
@@ -2113,8 +2302,12 @@
       <c r="H45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L45" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2012</v>
       </c>
@@ -2139,8 +2332,12 @@
       <c r="H46">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L46" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>2013</v>
       </c>
@@ -2165,8 +2362,12 @@
       <c r="H47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L47" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2014</v>
       </c>
@@ -2191,8 +2392,12 @@
       <c r="H48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L48" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2015</v>
       </c>
@@ -2217,8 +2422,12 @@
       <c r="H49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L49" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>2016</v>
       </c>
@@ -2246,8 +2455,12 @@
       <c r="I50">
         <v>2.202321724709785</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L50" s="3">
+        <f t="shared" si="0"/>
+        <v>2.2866982350408955</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>2017</v>
       </c>
@@ -2272,8 +2485,12 @@
       <c r="H51">
         <v>12319</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L51" s="3">
+        <f t="shared" si="0"/>
+        <v>1.0132659507264687</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>2018</v>
       </c>
@@ -2301,8 +2518,12 @@
       <c r="J52">
         <v>0.98571312606542738</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L52" s="3">
+        <f t="shared" si="0"/>
+        <v>0.59366680678156092</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>2019</v>
       </c>
@@ -2330,8 +2551,12 @@
       <c r="J53">
         <v>0.95310430786009193</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L53" s="3">
+        <f t="shared" si="0"/>
+        <v>0.53786322277663634</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>2020</v>
       </c>
@@ -2359,8 +2584,12 @@
       <c r="J54">
         <v>0.95364700410820868</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L54" s="3">
+        <f t="shared" si="0"/>
+        <v>0.5536673928830792</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>2021</v>
       </c>
@@ -2388,8 +2617,12 @@
       <c r="J55">
         <v>0.98467130214917831</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L55" s="3">
+        <f t="shared" si="0"/>
+        <v>0.56218402426693626</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>2022</v>
       </c>
@@ -2417,8 +2650,12 @@
       <c r="J56">
         <v>0.95447044704470452</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L56" s="3">
+        <f t="shared" si="0"/>
+        <v>0.52604096933993838</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>2023</v>
       </c>
@@ -2446,8 +2683,12 @@
       <c r="J57">
         <v>0.9835070095209536</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L57" s="3">
+        <f t="shared" si="0"/>
+        <v>0.80410297666934838</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>2010</v>
       </c>
@@ -2472,8 +2713,12 @@
       <c r="H58">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L58" s="3">
+        <f t="shared" si="0"/>
+        <v>1.5993715632364494</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>2011</v>
       </c>
@@ -2498,8 +2743,12 @@
       <c r="H59">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L59" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>2012</v>
       </c>
@@ -2524,8 +2773,12 @@
       <c r="H60">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L60" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>2013</v>
       </c>
@@ -2550,8 +2803,12 @@
       <c r="H61">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L61" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>2014</v>
       </c>
@@ -2576,8 +2833,12 @@
       <c r="H62">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L62" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>2015</v>
       </c>
@@ -2602,8 +2863,12 @@
       <c r="H63">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L63" s="3" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>2016</v>
       </c>
@@ -2631,8 +2896,12 @@
       <c r="I64">
         <v>2.2342342342342341</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L64" s="3">
+        <f t="shared" si="0"/>
+        <v>2.3279955825510767</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>2017</v>
       </c>
@@ -2657,8 +2926,12 @@
       <c r="H65">
         <v>9790</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L65" s="3">
+        <f t="shared" si="0"/>
+        <v>0.85313931554836975</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>2018</v>
       </c>
@@ -2686,8 +2959,12 @@
       <c r="J66">
         <v>0.9799795709908069</v>
       </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L66" s="3">
+        <f t="shared" si="0"/>
+        <v>0.35860582105641392</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>2019</v>
       </c>
@@ -2715,8 +2992,12 @@
       <c r="J67">
         <v>0.95498519249753211</v>
       </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L67" s="3">
+        <f t="shared" si="0"/>
+        <v>0.15861544313427159</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>2020</v>
       </c>
@@ -2744,8 +3025,12 @@
       <c r="J68">
         <v>0.95182740616688011</v>
       </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L68" s="3">
+        <f t="shared" ref="L68:L85" si="7">(E73+E74+E75)/(G67+G68+G69)</f>
+        <v>0.17146189735614309</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>2021</v>
       </c>
@@ -2773,8 +3058,12 @@
       <c r="J69">
         <v>0.98264664095798659</v>
       </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L69" s="3">
+        <f t="shared" si="7"/>
+        <v>0.18104133545310017</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>2022</v>
       </c>
@@ -2802,8 +3091,12 @@
       <c r="J70">
         <v>0.95611100177130481</v>
       </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L70" s="3">
+        <f t="shared" si="7"/>
+        <v>0.17401869158878505</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>2023</v>
       </c>
@@ -2831,8 +3124,12 @@
       <c r="J71">
         <v>0.98892878515858762</v>
       </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L71" s="3">
+        <f t="shared" si="7"/>
+        <v>0.26262626262626265</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>2010</v>
       </c>
@@ -2857,8 +3154,12 @@
       <c r="H72">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L72" s="3">
+        <f t="shared" si="7"/>
+        <v>0.51619989017023615</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>2011</v>
       </c>
@@ -2883,8 +3184,12 @@
       <c r="H73">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L73" s="3" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>2012</v>
       </c>
@@ -2909,8 +3214,12 @@
       <c r="H74">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L74" s="3" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>2013</v>
       </c>
@@ -2935,8 +3244,12 @@
       <c r="H75">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L75" s="3" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>2014</v>
       </c>
@@ -2961,8 +3274,12 @@
       <c r="H76">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L76" s="3" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>2015</v>
       </c>
@@ -2987,8 +3304,12 @@
       <c r="H77">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L77" s="3" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>2016</v>
       </c>
@@ -3016,8 +3337,12 @@
       <c r="I78">
         <v>2.087619047619047</v>
       </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L78" s="3">
+        <f t="shared" si="7"/>
+        <v>2.140625</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>2017</v>
       </c>
@@ -3042,8 +3367,12 @@
       <c r="H79">
         <v>2529</v>
       </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L79" s="3">
+        <f t="shared" si="7"/>
+        <v>0.94508670520231219</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>2018</v>
       </c>
@@ -3071,8 +3400,12 @@
       <c r="J80">
         <v>1.007908264136022</v>
       </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L80" s="3">
+        <f t="shared" si="7"/>
+        <v>0.77912157861234888</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>2019</v>
       </c>
@@ -3100,8 +3433,12 @@
       <c r="J81">
         <v>0.94606575544883631</v>
       </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L81" s="3">
+        <f t="shared" si="7"/>
+        <v>0.96786632390745497</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>2020</v>
       </c>
@@ -3129,8 +3466,12 @@
       <c r="J82">
         <v>0.96036363636363631</v>
       </c>
-    </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L82" s="3">
+        <f t="shared" si="7"/>
+        <v>1.1177484204480184</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>2021</v>
       </c>
@@ -3158,8 +3499,12 @@
       <c r="J83">
         <v>0.99179157744468238</v>
       </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L83" s="3">
+        <f t="shared" si="7"/>
+        <v>1.0269698572184029</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>2022</v>
       </c>
@@ -3187,8 +3532,12 @@
       <c r="J84">
         <v>0.94921135646687693</v>
       </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L84" s="3">
+        <f t="shared" si="7"/>
+        <v>0.93015573383671546</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>2023</v>
       </c>
@@ -3216,8 +3565,12 @@
       <c r="J85">
         <v>0.96709930576516756</v>
       </c>
-    </row>
-    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+      <c r="L85" s="3">
+        <f t="shared" si="7"/>
+        <v>0.7895962732919255</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>2010</v>
       </c>
@@ -3243,7 +3596,7 @@
         <v>5513</v>
       </c>
     </row>
-    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>2011</v>
       </c>
@@ -3275,7 +3628,7 @@
         <v>1.0545982223834569</v>
       </c>
     </row>
-    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>2012</v>
       </c>
@@ -3307,7 +3660,7 @@
         <v>1.0532158590308369</v>
       </c>
     </row>
-    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>2013</v>
       </c>
@@ -3339,7 +3692,7 @@
         <v>1.058586918502973</v>
       </c>
     </row>
-    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>2014</v>
       </c>
@@ -3371,7 +3724,7 @@
         <v>1.083928260491033</v>
       </c>
     </row>
-    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>2015</v>
       </c>
@@ -3403,7 +3756,7 @@
         <v>1.0248857287963431</v>
       </c>
     </row>
-    <row r="92" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>2016</v>
       </c>
@@ -3435,7 +3788,7 @@
         <v>1.061302681992337</v>
       </c>
     </row>
-    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>2017</v>
       </c>
@@ -3464,7 +3817,7 @@
         <v>1.000173701580684</v>
       </c>
     </row>
-    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>2018</v>
       </c>
@@ -3493,7 +3846,7 @@
         <v>1.09229098805646</v>
       </c>
     </row>
-    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>2019</v>
       </c>
@@ -3522,7 +3875,7 @@
         <v>1.038100301258196</v>
       </c>
     </row>
-    <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>2020</v>
       </c>
@@ -23124,7 +23477,7 @@
         <v>1.3419593345656191</v>
       </c>
     </row>
-    <row r="753" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="753" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A753">
         <v>2010</v>
       </c>
@@ -23149,8 +23502,12 @@
       <c r="H753">
         <v>0</v>
       </c>
-    </row>
-    <row r="754" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L753" s="3">
+        <f t="shared" ref="L753:L766" si="8">(E758+E759+E760)/(G752+G753+G754)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="754" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A754">
         <v>2011</v>
       </c>
@@ -23175,8 +23532,12 @@
       <c r="H754">
         <v>0</v>
       </c>
-    </row>
-    <row r="755" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L754" s="3" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="755" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A755">
         <v>2012</v>
       </c>
@@ -23201,8 +23562,12 @@
       <c r="H755">
         <v>0</v>
       </c>
-    </row>
-    <row r="756" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L755" s="3" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="756" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A756">
         <v>2013</v>
       </c>
@@ -23227,8 +23592,12 @@
       <c r="H756">
         <v>0</v>
       </c>
-    </row>
-    <row r="757" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L756" s="3" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="757" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A757">
         <v>2014</v>
       </c>
@@ -23253,8 +23622,12 @@
       <c r="H757">
         <v>0</v>
       </c>
-    </row>
-    <row r="758" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L757" s="3" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="758" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A758">
         <v>2015</v>
       </c>
@@ -23279,8 +23652,12 @@
       <c r="H758">
         <v>0</v>
       </c>
-    </row>
-    <row r="759" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L758" s="3" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="759" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A759">
         <v>2016</v>
       </c>
@@ -23308,8 +23685,12 @@
       <c r="I759">
         <v>14.96338028169014</v>
       </c>
-    </row>
-    <row r="760" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L759" s="3">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="760" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A760">
         <v>2017</v>
       </c>
@@ -23334,8 +23715,12 @@
       <c r="H760">
         <v>1443</v>
       </c>
-    </row>
-    <row r="761" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L760" s="3">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="761" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A761">
         <v>2018</v>
       </c>
@@ -23363,8 +23748,12 @@
       <c r="J761">
         <v>1.896742896742897</v>
       </c>
-    </row>
-    <row r="762" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L761" s="3">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="762" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A762">
         <v>2019</v>
       </c>
@@ -23392,8 +23781,12 @@
       <c r="J762">
         <v>1.743319268635724</v>
       </c>
-    </row>
-    <row r="763" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L762" s="3">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="763" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A763">
         <v>2020</v>
       </c>
@@ -23421,8 +23814,12 @@
       <c r="J763">
         <v>1.890472618154539</v>
       </c>
-    </row>
-    <row r="764" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L763" s="3">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="764" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A764">
         <v>2021</v>
       </c>
@@ -23450,8 +23847,12 @@
       <c r="J764">
         <v>1.902866242038217</v>
       </c>
-    </row>
-    <row r="765" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L764" s="3">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="765" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A765">
         <v>2022</v>
       </c>
@@ -23479,8 +23880,12 @@
       <c r="J765">
         <v>1.8924003009781789</v>
       </c>
-    </row>
-    <row r="766" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L765" s="3">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="766" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A766">
         <v>2023</v>
       </c>
@@ -23508,8 +23913,12 @@
       <c r="J766">
         <v>1.855835240274599</v>
       </c>
-    </row>
-    <row r="767" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+      <c r="L766" s="3">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="767" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A767">
         <v>2010</v>
       </c>
@@ -23535,7 +23944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="768" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="768" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A768">
         <v>2011</v>
       </c>

</xml_diff>

<commit_message>
updeted code duplication adressed WIP doing UNITID list
</commit_message>
<xml_diff>
--- a/PRC_National_dataset test.xlsx
+++ b/PRC_National_dataset test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/co25936/Desktop/PER/IPEDS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0965B8D-6A55-7D4A-A745-49BA67F819B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F07E75-945D-7340-B920-EF6B6650D513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="38400" windowHeight="17620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="17620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6646" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6679" uniqueCount="57">
   <si>
     <t>year</t>
   </si>
@@ -149,6 +149,66 @@
   <si>
     <t>TEST -&gt;</t>
   </si>
+  <si>
+    <t>IPEDS</t>
+  </si>
+  <si>
+    <t>UNITD</t>
+  </si>
+  <si>
+    <t>YEAR</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>MIP</t>
+  </si>
+  <si>
+    <t>Mip</t>
+  </si>
+  <si>
+    <t>2011 (INSTERTED)</t>
+  </si>
+  <si>
+    <t>GSS (2005)</t>
+  </si>
+  <si>
+    <t>GSS (2006)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPILE A TOTAL LIST OF UNITIDS AND FOR EACH ONE HAVE A ROW FOR EACH YEAR and fill out with apropitate data and then MIP </t>
+  </si>
+  <si>
+    <t>UNITID</t>
+  </si>
+  <si>
+    <t>FIRST</t>
+  </si>
+  <si>
+    <t>CTOTALT</t>
+  </si>
+  <si>
+    <t>AWLEVEL</t>
+  </si>
+  <si>
+    <t>Enrolled</t>
+  </si>
+  <si>
+    <t>2+4</t>
+  </si>
+  <si>
+    <t>6+4</t>
+  </si>
 </sst>
 </file>
 
@@ -219,13 +279,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -33032,10 +33093,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA2CE5D4-1C0B-B149-9B08-58F3451A04FC}">
-  <dimension ref="A1:R1107"/>
+  <dimension ref="A1:AD1107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -33076,7 +33137,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2010</v>
       </c>
@@ -33115,15 +33176,21 @@
         <v>0</v>
       </c>
       <c r="Q2">
-        <f t="shared" ref="P2:R17" si="0">L2-G2</f>
+        <f t="shared" ref="Q2:R17" si="0">L2-G2</f>
         <v>-67</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
         <v>-211</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V2" t="s">
+        <v>47</v>
+      </c>
+      <c r="W2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -33169,8 +33236,11 @@
         <f t="shared" si="0"/>
         <v>-280</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V3">
+        <v>81818128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2012</v>
       </c>
@@ -33217,7 +33287,7 @@
         <v>-205</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -33263,8 +33333,23 @@
         <f t="shared" si="0"/>
         <v>-151</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Y5" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -33310,8 +33395,23 @@
         <f t="shared" si="0"/>
         <v>-191</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Y6" s="2">
+        <v>194541</v>
+      </c>
+      <c r="Z6">
+        <v>2010</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2015</v>
       </c>
@@ -33357,8 +33457,23 @@
         <f t="shared" si="0"/>
         <v>-191</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Y7" s="2">
+        <v>194541</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2016</v>
       </c>
@@ -33404,8 +33519,26 @@
         <f t="shared" si="0"/>
         <v>-139</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V8" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y8" s="2">
+        <v>194541</v>
+      </c>
+      <c r="Z8">
+        <v>2012</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2017</v>
       </c>
@@ -33451,8 +33584,23 @@
         <f t="shared" si="0"/>
         <v>-79</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Y9" s="2">
+        <v>194541</v>
+      </c>
+      <c r="Z9">
+        <v>2013</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -33498,8 +33646,23 @@
         <f t="shared" si="0"/>
         <v>-78</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Y10" s="2">
+        <v>194541</v>
+      </c>
+      <c r="Z10">
+        <v>2015</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2019</v>
       </c>
@@ -33546,7 +33709,7 @@
         <v>-11</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -33593,7 +33756,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -33632,15 +33795,18 @@
         <v>0</v>
       </c>
       <c r="Q13">
-        <f t="shared" si="0"/>
+        <f>L13-G13</f>
         <v>0</v>
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -33687,7 +33853,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -33734,7 +33900,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2010</v>
       </c>
@@ -33781,7 +33947,7 @@
         <v>-166</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2011</v>
       </c>
@@ -33827,8 +33993,29 @@
         <f t="shared" si="0"/>
         <v>-225</v>
       </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V17" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="W17" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="X17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y17" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z17" s="4"/>
+      <c r="AA17" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB17" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC17" s="4"/>
+      <c r="AD17" s="4"/>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2012</v>
       </c>
@@ -33874,8 +34061,29 @@
         <f t="shared" si="2"/>
         <v>-153</v>
       </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V18" s="4">
+        <v>8182</v>
+      </c>
+      <c r="W18" s="4">
+        <v>7</v>
+      </c>
+      <c r="X18" s="4">
+        <v>2</v>
+      </c>
+      <c r="Y18" s="4">
+        <v>6</v>
+      </c>
+      <c r="Z18" s="4"/>
+      <c r="AA18" s="4">
+        <v>1</v>
+      </c>
+      <c r="AB18" s="4">
+        <v>2010</v>
+      </c>
+      <c r="AC18" s="4"/>
+      <c r="AD18" s="4"/>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2013</v>
       </c>
@@ -33921,8 +34129,29 @@
         <f t="shared" si="2"/>
         <v>-120</v>
       </c>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V19" s="4">
+        <v>8182</v>
+      </c>
+      <c r="W19" s="4">
+        <v>17</v>
+      </c>
+      <c r="X19" s="4">
+        <v>2</v>
+      </c>
+      <c r="Y19" s="4">
+        <v>6</v>
+      </c>
+      <c r="Z19" s="4"/>
+      <c r="AA19" s="4">
+        <v>4</v>
+      </c>
+      <c r="AB19" s="4">
+        <v>2010</v>
+      </c>
+      <c r="AC19" s="4"/>
+      <c r="AD19" s="4"/>
+    </row>
+    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2014</v>
       </c>
@@ -33968,8 +34197,29 @@
         <f t="shared" si="2"/>
         <v>-150</v>
       </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V20" s="4">
+        <v>8182</v>
+      </c>
+      <c r="W20" s="4">
+        <v>7</v>
+      </c>
+      <c r="X20" s="4">
+        <v>4</v>
+      </c>
+      <c r="Y20" s="4">
+        <v>4</v>
+      </c>
+      <c r="Z20" s="4"/>
+      <c r="AA20" s="4">
+        <v>3</v>
+      </c>
+      <c r="AB20" s="4">
+        <v>2011</v>
+      </c>
+      <c r="AC20" s="4"/>
+      <c r="AD20" s="4"/>
+    </row>
+    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2015</v>
       </c>
@@ -34015,8 +34265,25 @@
         <f t="shared" si="2"/>
         <v>-150</v>
       </c>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V21" s="4">
+        <v>8182</v>
+      </c>
+      <c r="W21" s="4">
+        <v>17</v>
+      </c>
+      <c r="X21" s="4">
+        <v>4</v>
+      </c>
+      <c r="Y21" s="4"/>
+      <c r="Z21" s="4"/>
+      <c r="AA21" s="4"/>
+      <c r="AB21" s="4">
+        <v>2012</v>
+      </c>
+      <c r="AC21" s="4"/>
+      <c r="AD21" s="4"/>
+    </row>
+    <row r="22" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2016</v>
       </c>
@@ -34062,8 +34329,25 @@
         <f t="shared" si="2"/>
         <v>-112</v>
       </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V22" s="4">
+        <v>8182</v>
+      </c>
+      <c r="W22" s="4">
+        <v>7</v>
+      </c>
+      <c r="X22" s="4">
+        <v>4</v>
+      </c>
+      <c r="Y22" s="4"/>
+      <c r="Z22" s="4"/>
+      <c r="AA22" s="4"/>
+      <c r="AB22" s="4">
+        <v>2012</v>
+      </c>
+      <c r="AC22" s="4"/>
+      <c r="AD22" s="4"/>
+    </row>
+    <row r="23" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2017</v>
       </c>
@@ -34109,8 +34393,17 @@
         <f t="shared" si="2"/>
         <v>-64</v>
       </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V23" s="4"/>
+      <c r="W23" s="4"/>
+      <c r="X23" s="4"/>
+      <c r="Y23" s="4"/>
+      <c r="Z23" s="4"/>
+      <c r="AA23" s="4"/>
+      <c r="AB23" s="4"/>
+      <c r="AC23" s="4"/>
+      <c r="AD23" s="4"/>
+    </row>
+    <row r="24" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2018</v>
       </c>
@@ -34156,8 +34449,17 @@
         <f t="shared" si="2"/>
         <v>-66</v>
       </c>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V24" s="4"/>
+      <c r="W24" s="4"/>
+      <c r="X24" s="4"/>
+      <c r="Y24" s="4"/>
+      <c r="Z24" s="4"/>
+      <c r="AA24" s="4"/>
+      <c r="AB24" s="4"/>
+      <c r="AC24" s="4"/>
+      <c r="AD24" s="4"/>
+    </row>
+    <row r="25" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2019</v>
       </c>
@@ -34203,8 +34505,21 @@
         <f t="shared" si="2"/>
         <v>-10</v>
       </c>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V25" s="4"/>
+      <c r="W25" s="4"/>
+      <c r="X25" s="4">
+        <v>2</v>
+      </c>
+      <c r="Y25" s="4">
+        <v>6</v>
+      </c>
+      <c r="Z25" s="4"/>
+      <c r="AA25" s="4"/>
+      <c r="AB25" s="4"/>
+      <c r="AC25" s="4"/>
+      <c r="AD25" s="4"/>
+    </row>
+    <row r="26" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2020</v>
       </c>
@@ -34250,8 +34565,21 @@
         <f t="shared" si="2"/>
         <v>-5</v>
       </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V26" s="4"/>
+      <c r="W26" s="4"/>
+      <c r="X26" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y26" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z26" s="4"/>
+      <c r="AA26" s="4"/>
+      <c r="AB26" s="4"/>
+      <c r="AC26" s="4"/>
+      <c r="AD26" s="4"/>
+    </row>
+    <row r="27" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2021</v>
       </c>
@@ -34297,8 +34625,21 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="V27" s="4"/>
+      <c r="W27" s="4"/>
+      <c r="X27" s="4">
+        <v>6</v>
+      </c>
+      <c r="Y27" s="4">
+        <v>10</v>
+      </c>
+      <c r="Z27" s="4"/>
+      <c r="AA27" s="4"/>
+      <c r="AB27" s="4"/>
+      <c r="AC27" s="4"/>
+      <c r="AD27" s="4"/>
+    </row>
+    <row r="28" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>2022</v>
       </c>
@@ -34345,7 +34686,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>2023</v>
       </c>
@@ -34392,7 +34733,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2010</v>
       </c>
@@ -34439,7 +34780,7 @@
         <v>-45</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>2011</v>
       </c>
@@ -34486,7 +34827,7 @@
         <v>-55</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>2012</v>
       </c>

</xml_diff>